<commit_message>
Spreadsheet plus checklist for steps
</commit_message>
<xml_diff>
--- a/Breakout.AI/Product-Hunt.xlsx
+++ b/Breakout.AI/Product-Hunt.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8160"/>
+    <workbookView windowWidth="22188" windowHeight="9000" firstSheet="3" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Product Hunt" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,9 @@
     <sheet name="UI Agentic Design Tools" sheetId="5" r:id="rId5"/>
     <sheet name="HealthCare AI Workflows" sheetId="6" r:id="rId6"/>
     <sheet name="Finalised Top picks" sheetId="7" r:id="rId7"/>
+    <sheet name="Reel-Generation" sheetId="8" r:id="rId8"/>
+    <sheet name="Tool-Stack" sheetId="9" r:id="rId9"/>
+    <sheet name="Comments" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="241">
   <si>
     <t>Priority</t>
   </si>
@@ -462,6 +465,300 @@
   </si>
   <si>
     <t>Therapy AI</t>
+  </si>
+  <si>
+    <t>Bob`s Reels</t>
+  </si>
+  <si>
+    <t>Complete Workflow recommendation with tools</t>
+  </si>
+  <si>
+    <t>Character:</t>
+  </si>
+  <si>
+    <t>Bob Campana</t>
+  </si>
+  <si>
+    <t>1. Video Generation(Images -&gt; clips)</t>
+  </si>
+  <si>
+    <t>Selected:</t>
+  </si>
+  <si>
+    <t>Story-Line-Two</t>
+  </si>
+  <si>
+    <t>1. Google flow</t>
+  </si>
+  <si>
+    <t>Story 1: The 1975 Hippie Trail and the Beirut War Zone Escape</t>
+  </si>
+  <si>
+    <t>2. Adobe Firefly</t>
+  </si>
+  <si>
+    <t>3. Runway Gen3</t>
+  </si>
+  <si>
+    <t>1. Grammar + Clarity Fix</t>
+  </si>
+  <si>
+    <t>4. Pika</t>
+  </si>
+  <si>
+    <t>Task-Assignment</t>
+  </si>
+  <si>
+    <t>Best Combo</t>
+  </si>
+  <si>
+    <t>1. Find the best AI video generation tools for creating 60-second reels from images.</t>
+  </si>
+  <si>
+    <t>1. Runway</t>
+  </si>
+  <si>
+    <t>2. Organize output in a Google Drive folder</t>
+  </si>
+  <si>
+    <t>2. Pika</t>
+  </si>
+  <si>
+    <t>3. Build a side project using MCP + RAG + LLM-based workflows</t>
+  </si>
+  <si>
+    <t>3. Firefly</t>
+  </si>
+  <si>
+    <t>4. Fully execute the workflow using selected tools.</t>
+  </si>
+  <si>
+    <t>5. Identify the best free tools for AI video generation(graphics + reels upto 60 seconds)</t>
+  </si>
+  <si>
+    <t>Background Music + Voice + Editing</t>
+  </si>
+  <si>
+    <t>Production Requirements</t>
+  </si>
+  <si>
+    <t>1. Capcut</t>
+  </si>
+  <si>
+    <t>2. Canva</t>
+  </si>
+  <si>
+    <t>1. Generate images first, then convert them into videos/reels.</t>
+  </si>
+  <si>
+    <t>3. DaVinci Resolve</t>
+  </si>
+  <si>
+    <t>2.Create 3-4 reels (each ~60 seconds).</t>
+  </si>
+  <si>
+    <t>3. Upload all outputs to a suitable "studio" or platform.</t>
+  </si>
+  <si>
+    <t>Storage / Google Folder</t>
+  </si>
+  <si>
+    <t>4. Maintain time intervals and compare tool performance.</t>
+  </si>
+  <si>
+    <t>Structure for submission:</t>
+  </si>
+  <si>
+    <t>5. Maintain time intervals and compare tool performance</t>
+  </si>
+  <si>
+    <t>/AI_Reels_Project</t>
+  </si>
+  <si>
+    <t>6. Ensure images are sequentially connected and numbered according to the script.</t>
+  </si>
+  <si>
+    <t>/Images</t>
+  </si>
+  <si>
+    <t>7. Add background music and narration/dialogue for each scene.</t>
+  </si>
+  <si>
+    <t>/Scene_Videos</t>
+  </si>
+  <si>
+    <t>8. Create short clips(5-10 seconds each) and merge them into a full reel.</t>
+  </si>
+  <si>
+    <t>/Final_Reels</t>
+  </si>
+  <si>
+    <t>9. Final output: 60 second video composed of mutliple scenes</t>
+  </si>
+  <si>
+    <t>/Audio</t>
+  </si>
+  <si>
+    <t>/Scripts</t>
+  </si>
+  <si>
+    <t>Note that reels should have:</t>
+  </si>
+  <si>
+    <t>1. Dialogues</t>
+  </si>
+  <si>
+    <t>2. Background Music</t>
+  </si>
+  <si>
+    <t>3. Captions</t>
+  </si>
+  <si>
+    <t>4. Made like an animated film</t>
+  </si>
+  <si>
+    <t>5. Prepare a character response sheet for Bob</t>
+  </si>
+  <si>
+    <t>Best AI Video Tool Stack</t>
+  </si>
+  <si>
+    <t>1. Main AI Video Generation</t>
+  </si>
+  <si>
+    <t>A. Runway Gen-3</t>
+  </si>
+  <si>
+    <t>B. Pika</t>
+  </si>
+  <si>
+    <t>C. Google Flow</t>
+  </si>
+  <si>
+    <t>2. Editing for 60seconds Reel</t>
+  </si>
+  <si>
+    <t>A. CapCut</t>
+  </si>
+  <si>
+    <t>1. Merge Clips</t>
+  </si>
+  <si>
+    <t>2. Add music</t>
+  </si>
+  <si>
+    <t>3. Add AI Voice narration</t>
+  </si>
+  <si>
+    <t>4. Transitions</t>
+  </si>
+  <si>
+    <t>5. Export 60-seconds reels</t>
+  </si>
+  <si>
+    <t>3. Image Generation</t>
+  </si>
+  <si>
+    <t>A. Adobe Firefly</t>
+  </si>
+  <si>
+    <t>1. Best for clean, professional visuals</t>
+  </si>
+  <si>
+    <t>B. Canva</t>
+  </si>
+  <si>
+    <t>1. Best for quick visuals + templates + beginners</t>
+  </si>
+  <si>
+    <t>4. Voice + Music</t>
+  </si>
+  <si>
+    <t>A. ElevenLabs</t>
+  </si>
+  <si>
+    <t>B. CapCut</t>
+  </si>
+  <si>
+    <t>1. Best tool for AI Gneneration video(60 seconds reel only) from images only !</t>
+  </si>
+  <si>
+    <t>2. Google folder also</t>
+  </si>
+  <si>
+    <t>3. Prepare side projects plus try to go with mcp plus RAG, LLM</t>
+  </si>
+  <si>
+    <t>4. Do these tools completely</t>
+  </si>
+  <si>
+    <t>5. best free tool for generating ai video generation graphics as well for 60 seconds reel generation</t>
+  </si>
+  <si>
+    <t>Task - Assignment</t>
+  </si>
+  <si>
+    <t>Charact</t>
+  </si>
+  <si>
+    <t>1. Please check the grammar of document, spelling mistakes, headings, font styles, font size.</t>
+  </si>
+  <si>
+    <t>2. Directly generate images and then make reel or videos of 60 seconds. (3-4)</t>
+  </si>
+  <si>
+    <t>3. upload all of these things in the studios whichever more better</t>
+  </si>
+  <si>
+    <t>4. Please keep the time interval ready made with comparision in between the options and choice provided.</t>
+  </si>
+  <si>
+    <t>5. All the images should adjacently connected to each other as numbered as per their scripts only.</t>
+  </si>
+  <si>
+    <t>6. Try to provide background music and and narrate specific dialogues for the scenes with this combination make a reel of 10 seconds and make video out of it</t>
+  </si>
+  <si>
+    <t>7. Step 5: Animate Each Scene</t>
+  </si>
+  <si>
+    <t>Most AI video tools currently generate short clips of around 5–10 seconds. Because of that,</t>
+  </si>
+  <si>
+    <t>create each 60-second reel by generating multiple short scenes and editing them together.</t>
+  </si>
+  <si>
+    <t>Recommended tools to test:</t>
+  </si>
+  <si>
+    <t>● Google Flow: https://labs.google/fx/tools/flow/</t>
+  </si>
+  <si>
+    <t>● Google Vids: https://vids.google.com/</t>
+  </si>
+  <si>
+    <t>● Adobe Firefly Video: https://firefly.adobe.com/generate/video</t>
+  </si>
+  <si>
+    <t>● Seedance or other AI video tools you discover</t>
+  </si>
+  <si>
+    <t>Tell me which tool to use for all functionalities:</t>
+  </si>
+  <si>
+    <t>1. Adding background music</t>
+  </si>
+  <si>
+    <t>2. Adding all the shorts from the range (5-10) seconds then merging all these ranges</t>
+  </si>
+  <si>
+    <t>3. Adding to make a 60 second reel from all the scene generated images</t>
+  </si>
+  <si>
+    <t>4. Adding one dialogue to the primary reel that has duration from (5-10) seconds</t>
+  </si>
+  <si>
+    <t>5.  Please list how to use prompts this way also</t>
   </si>
 </sst>
 </file>
@@ -1896,6 +2193,153 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="C3:C31"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="3" spans="3:3">
+      <c r="C3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="3:3">
+      <c r="C4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="5" spans="3:3">
+      <c r="C5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="3:3">
+      <c r="C6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="7" spans="3:3">
+      <c r="C7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3">
+      <c r="C9" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3">
+      <c r="C10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3">
+      <c r="C11" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="3:3">
+      <c r="C12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="3:3">
+      <c r="C13" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" spans="3:3">
+      <c r="C14" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="3:3">
+      <c r="C15" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16" spans="3:3">
+      <c r="C16" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3">
+      <c r="C29" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3">
+      <c r="C30" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="31" spans="3:3">
+      <c r="C31" t="s">
+        <v>240</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
@@ -2735,4 +3179,345 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:J37"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="18.4444444444444" customWidth="1"/>
+    <col min="2" max="2" width="22.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" t="s">
+        <v>149</v>
+      </c>
+      <c r="I4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="B5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="I6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="I9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>158</v>
+      </c>
+      <c r="I10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>160</v>
+      </c>
+      <c r="I11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>162</v>
+      </c>
+      <c r="I12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>165</v>
+      </c>
+      <c r="I14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>167</v>
+      </c>
+      <c r="I16" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="I17" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" t="s">
+        <v>170</v>
+      </c>
+      <c r="I18" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" t="s">
+        <v>173</v>
+      </c>
+      <c r="I20" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" t="s">
+        <v>175</v>
+      </c>
+      <c r="I21" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" t="s">
+        <v>177</v>
+      </c>
+      <c r="I22" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" t="s">
+        <v>179</v>
+      </c>
+      <c r="J23" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" t="s">
+        <v>181</v>
+      </c>
+      <c r="J24" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" t="s">
+        <v>183</v>
+      </c>
+      <c r="J25" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" t="s">
+        <v>185</v>
+      </c>
+      <c r="J26" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="J27" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="B32" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" t="s">
+        <v>193</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="B4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="B5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="B6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="B8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="C9" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="C10" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="C11" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="C12" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="C13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="B16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="C17" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="B18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="C19" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="B22" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="B23" t="s">
+        <v>213</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>